<commit_message>
more rules for header auto detection
</commit_message>
<xml_diff>
--- a/frontend/test_data/header_detection/Complex_Metadata_Test.xlsx
+++ b/frontend/test_data/header_detection/Complex_Metadata_Test.xlsx
@@ -498,7 +498,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:M7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -517,18 +517,27 @@
         <v>Consistent String Signal</v>
       </c>
       <c r="F1" t="str">
+        <v>Consistent Numeric Signal</v>
+      </c>
+      <c r="G1" t="str">
         <v>Pure Data Penalty</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
+        <v>Numeric Data Penalty</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Pivoted Series Bonus</v>
+      </c>
+      <c r="J1" t="str">
         <v>100% String Bonus</v>
       </c>
-      <c r="H1" t="str">
+      <c r="K1" t="str">
         <v>Unique Values Rule</v>
       </c>
-      <c r="I1" t="str">
+      <c r="L1" t="str">
         <v>Orphan Header Penalty</v>
       </c>
-      <c r="J1" t="str">
+      <c r="M1" t="str">
         <v>TOTAL SCORE</v>
       </c>
     </row>
@@ -552,15 +561,24 @@
         <v>0</v>
       </c>
       <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
         <v>10</v>
       </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
         <v>17</v>
       </c>
     </row>
@@ -584,15 +602,24 @@
         <v>0</v>
       </c>
       <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
         <v>10</v>
       </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-      <c r="J3">
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
         <v>17</v>
       </c>
     </row>
@@ -616,15 +643,24 @@
         <v>0</v>
       </c>
       <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
         <v>10</v>
       </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
         <v>17</v>
       </c>
     </row>
@@ -648,15 +684,24 @@
         <v>0</v>
       </c>
       <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
         <v>10</v>
       </c>
-      <c r="H5">
-        <v>0</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5">
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
         <v>17</v>
       </c>
     </row>
@@ -671,25 +716,34 @@
         <v>14</v>
       </c>
       <c r="D6">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="E6">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
       <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
         <v>10</v>
       </c>
-      <c r="H6">
+      <c r="K6">
         <v>5</v>
       </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-      <c r="J6">
-        <v>94</v>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>68</v>
       </c>
     </row>
     <row r="7">
@@ -706,7 +760,7 @@
         <v>0</v>
       </c>
       <c r="E7">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F7">
         <v>0</v>
@@ -715,18 +769,27 @@
         <v>0</v>
       </c>
       <c r="H7">
+        <v>-20</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
         <v>5</v>
       </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-      <c r="J7">
-        <v>39</v>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update header detection based on the keyword validation and imporving the Pivoted table rejection.
</commit_message>
<xml_diff>
--- a/frontend/test_data/header_detection/Complex_Metadata_Test.xlsx
+++ b/frontend/test_data/header_detection/Complex_Metadata_Test.xlsx
@@ -498,7 +498,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:N7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -508,37 +508,40 @@
         <v>Row Preview</v>
       </c>
       <c r="C1" t="str">
-        <v>Density Bonus</v>
+        <v>Pillar 1: Density (%)</v>
       </c>
       <c r="D1" t="str">
-        <v>Data Boundary Signal</v>
+        <v>Pillar 2: Boundary (%)</v>
       </c>
       <c r="E1" t="str">
-        <v>Consistent String Signal</v>
+        <v>Pillar 3: Consistency (%)</v>
       </c>
       <c r="F1" t="str">
-        <v>Consistent Numeric Signal</v>
+        <v>Pillar 4: Traits (%)</v>
       </c>
       <c r="G1" t="str">
         <v>Pure Data Penalty</v>
       </c>
       <c r="H1" t="str">
-        <v>Numeric Data Penalty</v>
+        <v>Mixed Data Penalty</v>
       </c>
       <c r="I1" t="str">
-        <v>Pivoted Series Bonus</v>
+        <v>Search Booster (Pivoted)</v>
       </c>
       <c r="J1" t="str">
-        <v>100% String Bonus</v>
+        <v>Orphan Header Penalty</v>
       </c>
       <c r="K1" t="str">
-        <v>Unique Values Rule</v>
+        <v>Duplicates Penalty</v>
       </c>
       <c r="L1" t="str">
-        <v>Orphan Header Penalty</v>
+        <v>FILLED CELLS</v>
       </c>
       <c r="M1" t="str">
-        <v>TOTAL SCORE</v>
+        <v>TOTAL RAW SCORE</v>
+      </c>
+      <c r="N1" t="str">
+        <v>NORMALIZED SCORE (%)</v>
       </c>
     </row>
     <row r="2">
@@ -549,16 +552,16 @@
         <v>["SMARTBRIDGE FINANCIAL EXPORT"]</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -570,16 +573,19 @@
         <v>0</v>
       </c>
       <c r="J2">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>0</v>
       </c>
       <c r="L2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M2">
-        <v>17</v>
+        <v>48</v>
+      </c>
+      <c r="N2">
+        <v>48</v>
       </c>
     </row>
     <row r="3">
@@ -590,16 +596,16 @@
         <v>["Generated On: 2026-06-13"]</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
       <c r="E3">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -611,16 +617,19 @@
         <v>0</v>
       </c>
       <c r="J3">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K3">
         <v>0</v>
       </c>
       <c r="L3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M3">
-        <v>17</v>
+        <v>48</v>
+      </c>
+      <c r="N3">
+        <v>48</v>
       </c>
     </row>
     <row r="4">
@@ -631,16 +640,16 @@
         <v>["Generated By: System Admin"]</v>
       </c>
       <c r="C4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4">
         <v>0</v>
       </c>
       <c r="E4">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -652,16 +661,19 @@
         <v>0</v>
       </c>
       <c r="J4">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K4">
         <v>0</v>
       </c>
       <c r="L4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M4">
-        <v>17</v>
+        <v>48</v>
+      </c>
+      <c r="N4">
+        <v>48</v>
       </c>
     </row>
     <row r="5">
@@ -672,16 +684,16 @@
         <v>["This report contains all vendor spend data for Q</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
       <c r="E5">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -693,16 +705,19 @@
         <v>0</v>
       </c>
       <c r="J5">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K5">
         <v>0</v>
       </c>
       <c r="L5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M5">
-        <v>17</v>
+        <v>48</v>
+      </c>
+      <c r="N5">
+        <v>48</v>
       </c>
     </row>
     <row r="6">
@@ -713,16 +728,16 @@
         <v>["Supplier ID","Supplier Name","City and State","N</v>
       </c>
       <c r="C6">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D6">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E6">
         <v>12</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -734,16 +749,19 @@
         <v>0</v>
       </c>
       <c r="J6">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K6">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L6">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="M6">
-        <v>68</v>
+        <v>73</v>
+      </c>
+      <c r="N6">
+        <v>73</v>
       </c>
     </row>
     <row r="7">
@@ -754,7 +772,7 @@
         <v>["S100","Initech","Austin TX","USA",50000,15,2000]</v>
       </c>
       <c r="C7">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -763,13 +781,13 @@
         <v>12</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G7">
         <v>0</v>
       </c>
       <c r="H7">
-        <v>-20</v>
+        <v>-30</v>
       </c>
       <c r="I7">
         <v>0</v>
@@ -778,18 +796,21 @@
         <v>0</v>
       </c>
       <c r="K7">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L7">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="M7">
-        <v>11</v>
+        <v>7</v>
+      </c>
+      <c r="N7">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Code improvement and validation logic improvement
</commit_message>
<xml_diff>
--- a/frontend/test_data/header_detection/Complex_Metadata_Test.xlsx
+++ b/frontend/test_data/header_detection/Complex_Metadata_Test.xlsx
@@ -498,7 +498,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:M7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -526,21 +526,18 @@
         <v>Mixed Data Penalty</v>
       </c>
       <c r="I1" t="str">
-        <v>Search Booster (Pivoted)</v>
+        <v>Orphan Header Penalty</v>
       </c>
       <c r="J1" t="str">
-        <v>Orphan Header Penalty</v>
+        <v>Duplicates Penalty</v>
       </c>
       <c r="K1" t="str">
-        <v>Duplicates Penalty</v>
+        <v>FILLED CELLS</v>
       </c>
       <c r="L1" t="str">
-        <v>FILLED CELLS</v>
+        <v>TOTAL RAW SCORE</v>
       </c>
       <c r="M1" t="str">
-        <v>TOTAL RAW SCORE</v>
-      </c>
-      <c r="N1" t="str">
         <v>NORMALIZED SCORE (%)</v>
       </c>
     </row>
@@ -576,15 +573,12 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L2">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="M2">
-        <v>48</v>
-      </c>
-      <c r="N2">
         <v>48</v>
       </c>
     </row>
@@ -620,15 +614,12 @@
         <v>0</v>
       </c>
       <c r="K3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="M3">
-        <v>48</v>
-      </c>
-      <c r="N3">
         <v>48</v>
       </c>
     </row>
@@ -664,15 +655,12 @@
         <v>0</v>
       </c>
       <c r="K4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L4">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="M4">
-        <v>48</v>
-      </c>
-      <c r="N4">
         <v>48</v>
       </c>
     </row>
@@ -708,15 +696,12 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L5">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="M5">
-        <v>48</v>
-      </c>
-      <c r="N5">
         <v>48</v>
       </c>
     </row>
@@ -752,15 +737,12 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L6">
-        <v>7</v>
+        <v>73</v>
       </c>
       <c r="M6">
-        <v>73</v>
-      </c>
-      <c r="N6">
         <v>73</v>
       </c>
     </row>
@@ -796,7 +778,7 @@
         <v>0</v>
       </c>
       <c r="K7">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L7">
         <v>7</v>
@@ -804,13 +786,10 @@
       <c r="M7">
         <v>7</v>
       </c>
-      <c r="N7">
-        <v>7</v>
-      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>